<commit_message>
Excel model: Sensitivity sheet (tariff vs capex, CUF and interest rate)
One-way tables of the tariff the target equity IRR needs, the equity IRR and the minimum DSCR at
the bid tariff with the capital cost, the solar and wind CUFs and the interest rate moved one at
a time, and two-way grids (capex × rate, capex × CUF, rate × CUF). Each point is a full run of the
app's financial model on the bid's inputs and energy, carried as the app's numbers (a tariff solved
for a target IRR is not one Excel formula); the base case is checked against the Live model on the
sheet. The in-app trace skips it. The feature list marks the sensitivity table live.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jKkuHBjiyJimAVAdehBdi
</commit_message>
<xml_diff>
--- a/docs/enterprise/FEATURES-JOULEWISE-CLIENT.xlsx
+++ b/docs/enterprise/FEATURES-JOULEWISE-CLIENT.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="390">
   <si>
     <t xml:space="preserve">TenderOS Enterprise: features by jouleWise and client responsibility</t>
   </si>
@@ -941,6 +941,9 @@
   </si>
   <si>
     <t xml:space="preserve">One-way and two-way sensitivities (tariff vs capex, CUF, rate) with the base case marked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Sensitivity sheet of the Excel model: one-way tables and two-way grids (capex, CUF, interest rate) from full runs of the model</t>
   </si>
   <si>
     <t xml:space="preserve">W-04</t>
@@ -4128,7 +4131,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
         <v>302</v>
       </c>
@@ -4148,7 +4151,7 @@
         <v>123</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>107</v>
+        <v>42</v>
       </c>
       <c r="H63" s="5" t="s">
         <v>61</v>
@@ -4159,20 +4162,22 @@
       <c r="J63" s="9" t="s">
         <v>296</v>
       </c>
-      <c r="K63" s="7"/>
+      <c r="K63" s="7" t="s">
+        <v>305</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>292</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E64" s="5" t="s">
         <v>78</v>
@@ -4193,21 +4198,21 @@
         <v>296</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E65" s="5" t="s">
         <v>78</v>
@@ -4222,27 +4227,27 @@
         <v>43</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J65" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K65" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E66" s="5" t="s">
         <v>78</v>
@@ -4257,27 +4262,27 @@
         <v>43</v>
       </c>
       <c r="I66" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J66" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>78</v>
@@ -4292,25 +4297,25 @@
         <v>43</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J67" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K67" s="7"/>
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E68" s="5" t="s">
         <v>78</v>
@@ -4325,25 +4330,25 @@
         <v>43</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J68" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K68" s="7"/>
     </row>
     <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E69" s="5" t="s">
         <v>147</v>
@@ -4358,25 +4363,25 @@
         <v>43</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J69" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K69" s="7"/>
     </row>
     <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E70" s="5" t="s">
         <v>114</v>
@@ -4391,27 +4396,27 @@
         <v>61</v>
       </c>
       <c r="I70" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J70" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K70" s="7" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>78</v>
@@ -4426,25 +4431,25 @@
         <v>61</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J71" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K71" s="7"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>114</v>
@@ -4459,25 +4464,25 @@
         <v>43</v>
       </c>
       <c r="I72" s="8" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J72" s="9" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K72" s="7"/>
     </row>
     <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>114</v>
@@ -4492,25 +4497,25 @@
         <v>61</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J73" s="9" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K73" s="7"/>
     </row>
     <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>114</v>
@@ -4525,27 +4530,27 @@
         <v>43</v>
       </c>
       <c r="I74" s="8" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J74" s="9" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>114</v>
@@ -4560,27 +4565,27 @@
         <v>43</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J75" s="9" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="K75" s="7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>114</v>
@@ -4595,27 +4600,27 @@
         <v>43</v>
       </c>
       <c r="I76" s="8" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J76" s="9" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K76" s="7" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E77" s="5" t="s">
         <v>114</v>
@@ -4630,25 +4635,25 @@
         <v>43</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J77" s="9" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K77" s="7"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D78" s="7" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E78" s="5" t="s">
         <v>78</v>
@@ -4663,25 +4668,25 @@
         <v>96</v>
       </c>
       <c r="I78" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="J78" s="9" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="K78" s="7"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>114</v>
@@ -4696,13 +4701,13 @@
         <v>96</v>
       </c>
       <c r="I79" s="8" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J79" s="9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K79" s="7" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
@@ -4753,7 +4758,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4770,7 +4775,7 @@
         <v>107</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4884,7 +4889,7 @@
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A9,Features!$G$2:$G$79,"Live")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A9,Features!$G$2:$G$79,"Extend")</f>
@@ -4892,7 +4897,7 @@
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A9,Features!$G$2:$G$79,"Build")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="13" t="n">
         <f aca="false">SUM(B9:D9)</f>
@@ -4901,7 +4906,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A10,Features!$G$2:$G$79,"Live")</f>
@@ -4922,7 +4927,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A11,Features!$G$2:$G$79,"Live")</f>
@@ -4943,11 +4948,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B12" s="15" t="n">
         <f aca="false">SUM(B4:B11)</f>
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C12" s="15" t="n">
         <f aca="false">SUM(C4:C11)</f>
@@ -4955,7 +4960,7 @@
       </c>
       <c r="D12" s="15" t="n">
         <f aca="false">SUM(D4:D11)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E12" s="15" t="n">
         <f aca="false">SUM(E4:E11)</f>
@@ -4964,7 +4969,7 @@
     </row>
     <row r="14" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4972,13 +4977,13 @@
         <v>18</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>42</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5025,11 +5030,11 @@
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A19,Features!$G$2:$G$79,"Live")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D19" s="13" t="n">
         <f aca="false">B19-C19</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5102,7 +5107,7 @@
     </row>
     <row r="25" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5110,7 +5115,7 @@
         <v>33</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -5121,7 +5126,7 @@
         <v>34</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>

</xml_diff>

<commit_message>
Feedback on any section and the Change requests tab, exported as a prompt for Claude Code
Give feedback (sidebar) outlines the section under the mouse on any page; a click opens a note that
is saved as a change request with where it was raised (tab, step, section, the boxes in it), who
and when. Change requests lists them with approve / reject (super admin), and "Export approved as a
prompt (.md)" downloads one Markdown file holding the instructions for Claude Code, every approved
request with its context and the code it touches, and a code map; the requests become Exported with
the batch, and Done once the change ships. Migration 013; check of the prompt; a browser test that
raises, approves, exports and reads the file back.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jKkuHBjiyJimAVAdehBdi
</commit_message>
<xml_diff>
--- a/docs/enterprise/FEATURES-JOULEWISE-CLIENT.xlsx
+++ b/docs/enterprise/FEATURES-JOULEWISE-CLIENT.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Features!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Features!$A$1:$K$79</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Features!$A$1:$K$80</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="394">
   <si>
     <t xml:space="preserve">TenderOS Enterprise: features by jouleWise and client responsibility</t>
   </si>
@@ -982,6 +982,18 @@
     <t xml:space="preserve">E-02</t>
   </si>
   <si>
+    <t xml:space="preserve">Feedback and change requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Give feedback: click any section of any page and write what should change; the Change requests tab lists every request (when, where, comment, by which team) with approve / reject; the approved ones export as one Markdown prompt for jouleWise to apply with Claude Code under the AMC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">web/src/feedback; tests/e2e/test_feedback.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-03</t>
+  </si>
+  <si>
     <t xml:space="preserve">Evidence status on every box</t>
   </si>
   <si>
@@ -991,7 +1003,7 @@
     <t xml:space="preserve">Faint / with count / signed off at this value / signed at an older value; the register as CSV</t>
   </si>
   <si>
-    <t xml:space="preserve">E-03</t>
+    <t xml:space="preserve">E-04</t>
   </si>
   <si>
     <t xml:space="preserve">Assignments</t>
@@ -1000,7 +1012,7 @@
     <t xml:space="preserve">A data point assigned to a team or person; answer with a value, note or file; accept or return into the bid as a new version</t>
   </si>
   <si>
-    <t xml:space="preserve">E-04</t>
+    <t xml:space="preserve">E-05</t>
   </si>
   <si>
     <t xml:space="preserve">Pings from any box (@mentions)</t>
@@ -1009,7 +1021,7 @@
     <t xml:space="preserve">A thread on every input box; mention a teammate; reply with a value; Fill in</t>
   </si>
   <si>
-    <t xml:space="preserve">E-05</t>
+    <t xml:space="preserve">E-06</t>
   </si>
   <si>
     <t xml:space="preserve">Team setup</t>
@@ -1018,7 +1030,7 @@
     <t xml:space="preserve">People, teams, super admin, titles, the tabs they cover</t>
   </si>
   <si>
-    <t xml:space="preserve">E-06</t>
+    <t xml:space="preserve">E-07</t>
   </si>
   <si>
     <t xml:space="preserve">Activity and audit log</t>
@@ -1030,7 +1042,7 @@
     <t xml:space="preserve">Activity log today; export to build</t>
   </si>
   <si>
-    <t xml:space="preserve">E-07</t>
+    <t xml:space="preserve">E-08</t>
   </si>
   <si>
     <t xml:space="preserve">Email notifications</t>
@@ -1999,7 +2011,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -4236,7 +4248,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
         <v>317</v>
       </c>
@@ -4302,20 +4314,22 @@
       <c r="J67" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="K67" s="7"/>
+      <c r="K67" s="7" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>311</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E68" s="5" t="s">
         <v>78</v>
@@ -4339,19 +4353,19 @@
     </row>
     <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>311</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>147</v>
+        <v>78</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>123</v>
@@ -4372,28 +4386,28 @@
     </row>
     <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>311</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>123</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="H70" s="5" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="I70" s="8" t="s">
         <v>314</v>
@@ -4401,9 +4415,7 @@
       <c r="J70" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="K70" s="7" t="s">
-        <v>333</v>
-      </c>
+      <c r="K70" s="7"/>
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
@@ -4419,13 +4431,13 @@
         <v>336</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="F71" s="5" t="s">
         <v>123</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="H71" s="5" t="s">
         <v>61</v>
@@ -4436,14 +4448,16 @@
       <c r="J71" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="K71" s="7"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K71" s="7" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>338</v>
+        <v>311</v>
       </c>
       <c r="C72" s="7" t="s">
         <v>339</v>
@@ -4452,70 +4466,70 @@
         <v>340</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G72" s="5" t="s">
         <v>42</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="I72" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="J72" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="K72" s="7"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="J72" s="9" t="s">
+      <c r="B73" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="K72" s="7"/>
-    </row>
-    <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="5" t="s">
+      <c r="C73" s="7" t="s">
         <v>343</v>
       </c>
-      <c r="B73" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C73" s="7" t="s">
+      <c r="D73" s="7" t="s">
         <v>344</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>345</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>114</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>107</v>
+        <v>42</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="I73" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="J73" s="9" t="s">
         <v>346</v>
       </c>
-      <c r="J73" s="9" t="s">
+      <c r="K73" s="7"/>
+    </row>
+    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="K73" s="7"/>
-    </row>
-    <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="5" t="s">
+      <c r="B74" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C74" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="B74" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C74" s="7" t="s">
+      <c r="D74" s="7" t="s">
         <v>349</v>
-      </c>
-      <c r="D74" s="7" t="s">
-        <v>350</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>114</v>
@@ -4524,33 +4538,31 @@
         <v>123</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>42</v>
+        <v>107</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="I74" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="J74" s="9" t="s">
         <v>351</v>
       </c>
-      <c r="J74" s="9" t="s">
+      <c r="K74" s="7"/>
+    </row>
+    <row r="75" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="K74" s="7" t="s">
+      <c r="B75" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C75" s="7" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="75" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="5" t="s">
+      <c r="D75" s="7" t="s">
         <v>354</v>
-      </c>
-      <c r="B75" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C75" s="7" t="s">
-        <v>355</v>
-      </c>
-      <c r="D75" s="7" t="s">
-        <v>356</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>114</v>
@@ -4565,27 +4577,27 @@
         <v>43</v>
       </c>
       <c r="I75" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="J75" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="K75" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="J75" s="9" t="s">
+    </row>
+    <row r="76" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="K75" s="7" t="s">
+      <c r="B76" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C76" s="7" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="5" t="s">
+      <c r="D76" s="7" t="s">
         <v>360</v>
-      </c>
-      <c r="B76" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C76" s="7" t="s">
-        <v>361</v>
-      </c>
-      <c r="D76" s="7" t="s">
-        <v>362</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>114</v>
@@ -4600,33 +4612,33 @@
         <v>43</v>
       </c>
       <c r="I76" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="J76" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="K76" s="7" t="s">
         <v>363</v>
-      </c>
-      <c r="J76" s="9" t="s">
-        <v>364</v>
-      </c>
-      <c r="K76" s="7" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="D77" s="7" t="s">
         <v>366</v>
-      </c>
-      <c r="B77" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C77" s="7" t="s">
-        <v>367</v>
-      </c>
-      <c r="D77" s="7" t="s">
-        <v>368</v>
       </c>
       <c r="E77" s="5" t="s">
         <v>114</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G77" s="5" t="s">
         <v>42</v>
@@ -4635,28 +4647,30 @@
         <v>43</v>
       </c>
       <c r="I77" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="J77" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="K77" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="J77" s="9" t="s">
+    </row>
+    <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="K77" s="7"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="5" t="s">
+      <c r="B78" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C78" s="7" t="s">
         <v>371</v>
       </c>
-      <c r="B78" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C78" s="7" t="s">
+      <c r="D78" s="7" t="s">
         <v>372</v>
       </c>
-      <c r="D78" s="7" t="s">
-        <v>373</v>
-      </c>
       <c r="E78" s="5" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="F78" s="5" t="s">
         <v>115</v>
@@ -4665,34 +4679,34 @@
         <v>42</v>
       </c>
       <c r="H78" s="5" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="I78" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="J78" s="9" t="s">
         <v>374</v>
-      </c>
-      <c r="J78" s="9" t="s">
-        <v>375</v>
       </c>
       <c r="K78" s="7"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C79" s="7" t="s">
         <v>376</v>
       </c>
-      <c r="B79" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="C79" s="7" t="s">
+      <c r="D79" s="7" t="s">
         <v>377</v>
       </c>
-      <c r="D79" s="7" t="s">
-        <v>378</v>
-      </c>
       <c r="E79" s="5" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>41</v>
+        <v>115</v>
       </c>
       <c r="G79" s="5" t="s">
         <v>42</v>
@@ -4701,18 +4715,51 @@
         <v>96</v>
       </c>
       <c r="I79" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="J79" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="J79" s="9" t="s">
+      <c r="K79" s="7"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="K79" s="7" t="s">
+      <c r="B80" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C80" s="7" t="s">
         <v>381</v>
       </c>
+      <c r="D80" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G80" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H80" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="I80" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="J80" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="K80" s="7" t="s">
+        <v>385</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K79"/>
-  <conditionalFormatting sqref="G2:G79">
+  <autoFilter ref="A1:K80"/>
+  <conditionalFormatting sqref="G2:G80">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$G2="Live"</formula>
     </cfRule>
@@ -4724,11 +4771,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" error="One of Live, Extend, Build" errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G79" type="list">
+    <dataValidation allowBlank="false" error="One of Live, Extend, Build" errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G80" type="list">
       <formula1>"Live,Extend,Build"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="One of P1, P2, P3" errorStyle="stop" errorTitle="Priority" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H79" type="list">
+    <dataValidation allowBlank="false" error="One of P1, P2, P3" errorStyle="stop" errorTitle="Priority" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H80" type="list">
       <formula1>"P1,P2,P3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4758,7 +4805,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4775,7 +4822,7 @@
         <v>107</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4783,15 +4830,15 @@
         <v>37</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A4,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A4,Features!$G$2:$G$80,"Live")</f>
         <v>13</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A4,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A4,Features!$G$2:$G$80,"Extend")</f>
         <v>2</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A4,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A4,Features!$G$2:$G$80,"Build")</f>
         <v>2</v>
       </c>
       <c r="E4" s="13" t="n">
@@ -4804,15 +4851,15 @@
         <v>120</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A5,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A5,Features!$G$2:$G$80,"Live")</f>
         <v>8</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A5,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A5,Features!$G$2:$G$80,"Extend")</f>
         <v>0</v>
       </c>
       <c r="D5" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A5,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A5,Features!$G$2:$G$80,"Build")</f>
         <v>1</v>
       </c>
       <c r="E5" s="13" t="n">
@@ -4825,15 +4872,15 @@
         <v>162</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A6,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A6,Features!$G$2:$G$80,"Live")</f>
         <v>12</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A6,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A6,Features!$G$2:$G$80,"Extend")</f>
         <v>0</v>
       </c>
       <c r="D6" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A6,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A6,Features!$G$2:$G$80,"Build")</f>
         <v>0</v>
       </c>
       <c r="E6" s="13" t="n">
@@ -4846,15 +4893,15 @@
         <v>212</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A7,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A7,Features!$G$2:$G$80,"Live")</f>
         <v>6</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A7,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A7,Features!$G$2:$G$80,"Extend")</f>
         <v>0</v>
       </c>
       <c r="D7" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A7,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A7,Features!$G$2:$G$80,"Build")</f>
         <v>0</v>
       </c>
       <c r="E7" s="13" t="n">
@@ -4867,15 +4914,15 @@
         <v>95</v>
       </c>
       <c r="B8" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A8,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A8,Features!$G$2:$G$80,"Live")</f>
         <v>15</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A8,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A8,Features!$G$2:$G$80,"Extend")</f>
         <v>0</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A8,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A8,Features!$G$2:$G$80,"Build")</f>
         <v>0</v>
       </c>
       <c r="E8" s="13" t="n">
@@ -4888,15 +4935,15 @@
         <v>292</v>
       </c>
       <c r="B9" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A9,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A9,Features!$G$2:$G$80,"Live")</f>
         <v>3</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A9,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A9,Features!$G$2:$G$80,"Extend")</f>
         <v>1</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A9,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A9,Features!$G$2:$G$80,"Build")</f>
         <v>0</v>
       </c>
       <c r="E9" s="13" t="n">
@@ -4909,36 +4956,36 @@
         <v>311</v>
       </c>
       <c r="B10" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A10,Features!$G$2:$G$79,"Live")</f>
-        <v>6</v>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A10,Features!$G$2:$G$80,"Live")</f>
+        <v>7</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A10,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A10,Features!$G$2:$G$80,"Extend")</f>
         <v>1</v>
       </c>
       <c r="D10" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A10,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A10,Features!$G$2:$G$80,"Build")</f>
         <v>0</v>
       </c>
       <c r="E10" s="13" t="n">
         <f aca="false">SUM(B10:D10)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B11" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A11,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A11,Features!$G$2:$G$80,"Live")</f>
         <v>7</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A11,Features!$G$2:$G$79,"Extend")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A11,Features!$G$2:$G$80,"Extend")</f>
         <v>0</v>
       </c>
       <c r="D11" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$B$2:$B$79,$A11,Features!$G$2:$G$79,"Build")</f>
+        <f aca="false">COUNTIFS(Features!$B$2:$B$80,$A11,Features!$G$2:$G$80,"Build")</f>
         <v>1</v>
       </c>
       <c r="E11" s="13" t="n">
@@ -4948,11 +4995,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B12" s="15" t="n">
         <f aca="false">SUM(B4:B11)</f>
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C12" s="15" t="n">
         <f aca="false">SUM(C4:C11)</f>
@@ -4964,12 +5011,12 @@
       </c>
       <c r="E12" s="15" t="n">
         <f aca="false">SUM(E4:E11)</f>
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4977,13 +5024,13 @@
         <v>18</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>42</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4991,11 +5038,11 @@
         <v>40</v>
       </c>
       <c r="B17" s="13" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$79,$A17)</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$80,$A17)</f>
         <v>14</v>
       </c>
       <c r="C17" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A17,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$E$2:$E$80,$A17,Features!$G$2:$G$80,"Live")</f>
         <v>13</v>
       </c>
       <c r="D17" s="13" t="n">
@@ -5008,12 +5055,12 @@
         <v>78</v>
       </c>
       <c r="B18" s="13" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$79,$A18)</f>
-        <v>15</v>
+        <f aca="false">COUNTIF(Features!$E$2:$E$80,$A18)</f>
+        <v>16</v>
       </c>
       <c r="C18" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A18,Features!$G$2:$G$79,"Live")</f>
-        <v>12</v>
+        <f aca="false">COUNTIFS(Features!$E$2:$E$80,$A18,Features!$G$2:$G$80,"Live")</f>
+        <v>13</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">B18-C18</f>
@@ -5025,11 +5072,11 @@
         <v>95</v>
       </c>
       <c r="B19" s="13" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$79,$A19)</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$80,$A19)</f>
         <v>18</v>
       </c>
       <c r="C19" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A19,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$E$2:$E$80,$A19,Features!$G$2:$G$80,"Live")</f>
         <v>18</v>
       </c>
       <c r="D19" s="13" t="n">
@@ -5042,11 +5089,11 @@
         <v>114</v>
       </c>
       <c r="B20" s="13" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$79,$A20)</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$80,$A20)</f>
         <v>9</v>
       </c>
       <c r="C20" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A20,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$E$2:$E$80,$A20,Features!$G$2:$G$80,"Live")</f>
         <v>6</v>
       </c>
       <c r="D20" s="13" t="n">
@@ -5059,11 +5106,11 @@
         <v>134</v>
       </c>
       <c r="B21" s="13" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$79,$A21)</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$80,$A21)</f>
         <v>3</v>
       </c>
       <c r="C21" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A21,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$E$2:$E$80,$A21,Features!$G$2:$G$80,"Live")</f>
         <v>3</v>
       </c>
       <c r="D21" s="13" t="n">
@@ -5076,11 +5123,11 @@
         <v>147</v>
       </c>
       <c r="B22" s="13" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$79,$A22)</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$80,$A22)</f>
         <v>5</v>
       </c>
       <c r="C22" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A22,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$E$2:$E$80,$A22,Features!$G$2:$G$80,"Live")</f>
         <v>4</v>
       </c>
       <c r="D22" s="13" t="n">
@@ -5093,11 +5140,11 @@
         <v>162</v>
       </c>
       <c r="B23" s="13" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$79,$A23)</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$80,$A23)</f>
         <v>14</v>
       </c>
       <c r="C23" s="13" t="n">
-        <f aca="false">COUNTIFS(Features!$E$2:$E$79,$A23,Features!$G$2:$G$79,"Live")</f>
+        <f aca="false">COUNTIFS(Features!$E$2:$E$80,$A23,Features!$G$2:$G$80,"Live")</f>
         <v>14</v>
       </c>
       <c r="D23" s="13" t="n">
@@ -5107,7 +5154,7 @@
     </row>
     <row r="25" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5115,7 +5162,7 @@
         <v>33</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -5126,7 +5173,7 @@
         <v>34</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>

</xml_diff>